<commit_message>
Updated v1.0 testing to fix camera test power typo
</commit_message>
<xml_diff>
--- a/Testing/C2Sv1/SYSTEM/Data.xlsx
+++ b/Testing/C2Sv1/SYSTEM/Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Felix\Desktop\C2S-software (2)\C2S-software\Testing\C2Sv1\SYSTEM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\C2S\Testing\C2Sv1\SYSTEM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E7A9872-C827-4C83-B771-0F8E6868E19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBBBD5F-01B7-4167-A2E7-D7E1C28045F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-1872" windowWidth="30936" windowHeight="16776" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SYS INFO" sheetId="2" r:id="rId1"/>
@@ -838,17 +838,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D5221BD-7002-446A-8FF9-DEDB49D8BCE4}">
   <dimension ref="B2:F11"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="2"/>
-    <col min="2" max="2" width="34.44140625" style="2" customWidth="1"/>
-    <col min="3" max="4" width="12.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="33.5546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="74.6640625" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="2"/>
+    <col min="1" max="1" width="9.140625" style="2"/>
+    <col min="2" max="2" width="34.42578125" style="2" customWidth="1"/>
+    <col min="3" max="4" width="12.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="33.5703125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="74.7109375" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
@@ -865,7 +865,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" ht="15" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
@@ -880,7 +880,7 @@
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" ht="15" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
@@ -893,7 +893,7 @@
       <c r="E4" s="3"/>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" ht="15" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
@@ -906,7 +906,7 @@
       <c r="E5" s="3"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" ht="15" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
@@ -921,7 +921,7 @@
       </c>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" ht="15" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
@@ -938,7 +938,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" ht="15" x14ac:dyDescent="0.2">
       <c r="B8" s="1" t="s">
         <v>76</v>
       </c>
@@ -952,7 +952,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" ht="15" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
         <v>78</v>
       </c>
@@ -966,7 +966,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B11" s="15" t="s">
         <v>67</v>
       </c>
@@ -979,25 +979,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:N38"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="2"/>
+    <col min="1" max="1" width="9.140625" style="2"/>
     <col min="2" max="2" width="9" style="2" customWidth="1"/>
-    <col min="3" max="3" width="22.88671875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="21.5546875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" style="2"/>
-    <col min="6" max="6" width="7.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.88671875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="22.44140625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" style="2"/>
-    <col min="10" max="10" width="9.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.33203125" style="2" customWidth="1"/>
-    <col min="12" max="13" width="9.109375" style="2"/>
-    <col min="14" max="14" width="20.6640625" style="2" customWidth="1"/>
-    <col min="15" max="16384" width="9.109375" style="2"/>
+    <col min="3" max="3" width="22.85546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="21.5703125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="2"/>
+    <col min="6" max="6" width="7.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.85546875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="22.42578125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="2"/>
+    <col min="10" max="10" width="9.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.28515625" style="2" customWidth="1"/>
+    <col min="12" max="13" width="9.140625" style="2"/>
+    <col min="14" max="14" width="20.7109375" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:14" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="25" t="s">
         <v>24</v>
       </c>
@@ -1016,7 +1016,7 @@
       <c r="M2" s="26"/>
       <c r="N2" s="26"/>
     </row>
-    <row r="3" spans="2:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
         <v>0</v>
       </c>
@@ -1048,7 +1048,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B4" s="3">
         <v>1</v>
       </c>
@@ -1082,7 +1082,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B5" s="3">
         <v>2</v>
       </c>
@@ -1116,7 +1116,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B6" s="3">
         <v>3</v>
       </c>
@@ -1150,7 +1150,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B7" s="3">
         <v>4</v>
       </c>
@@ -1184,7 +1184,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B8" s="3">
         <v>5</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.2">
       <c r="J9" s="3">
         <v>6</v>
       </c>
@@ -1232,7 +1232,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" ht="15" x14ac:dyDescent="0.2">
       <c r="C10" s="6" t="s">
         <v>12</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.2">
       <c r="J11" s="3">
         <v>8</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.2">
       <c r="J12" s="3">
         <v>9</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.2">
       <c r="J13" s="3">
         <v>10</v>
       </c>
@@ -1302,7 +1302,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
       <c r="J14" s="3">
         <v>11</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.2">
       <c r="J15" s="3">
         <v>12</v>
       </c>
@@ -1330,7 +1330,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" x14ac:dyDescent="0.2">
       <c r="J16" s="3">
         <v>13</v>
       </c>
@@ -1344,7 +1344,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="17" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J17" s="3">
         <v>14</v>
       </c>
@@ -1358,7 +1358,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="18" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J18" s="3">
         <v>15</v>
       </c>
@@ -1372,7 +1372,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="19" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J19" s="3">
         <v>16</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="20" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J20" s="3">
         <v>17</v>
       </c>
@@ -1400,7 +1400,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="21" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J21" s="3">
         <v>18</v>
       </c>
@@ -1414,7 +1414,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="22" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J22" s="3">
         <v>19</v>
       </c>
@@ -1428,7 +1428,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="23" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J23" s="3">
         <v>20</v>
       </c>
@@ -1442,7 +1442,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J24" s="3">
         <v>21</v>
       </c>
@@ -1456,7 +1456,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="25" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J25" s="3">
         <v>22</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="26" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J26" s="3">
         <v>23</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="27" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J27" s="3">
         <v>24</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="28" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J28" s="3">
         <v>25</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="30" spans="10:14" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="30" spans="10:14" ht="30" x14ac:dyDescent="0.2">
       <c r="J30" s="6" t="s">
         <v>12</v>
       </c>
@@ -1528,27 +1528,27 @@
         <v>150.68</v>
       </c>
     </row>
-    <row r="32" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J32" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="33" spans="10:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J33" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="10:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J35" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="10:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J36" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="38" spans="10:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J38" s="2" t="s">
         <v>80</v>
       </c>
@@ -1566,33 +1566,33 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCB63DF8-6718-44FD-B74D-334594AAEDEC}">
   <dimension ref="B2:W114"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="11"/>
-    <col min="2" max="2" width="13.33203125" style="11" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" style="11" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" style="11" customWidth="1"/>
-    <col min="8" max="8" width="17.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.6640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.6640625" style="11" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" style="11" customWidth="1"/>
-    <col min="12" max="12" width="14.6640625" style="11" customWidth="1"/>
-    <col min="13" max="13" width="9.109375" style="11"/>
-    <col min="14" max="14" width="11.6640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.88671875" style="11" customWidth="1"/>
-    <col min="16" max="16" width="9.109375" style="11"/>
-    <col min="17" max="17" width="11.6640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.88671875" style="11" customWidth="1"/>
-    <col min="19" max="21" width="9.109375" style="11"/>
-    <col min="22" max="22" width="12.109375" style="11" customWidth="1"/>
-    <col min="23" max="23" width="14.109375" style="11" customWidth="1"/>
-    <col min="24" max="16384" width="9.109375" style="11"/>
+    <col min="1" max="1" width="9.140625" style="11"/>
+    <col min="2" max="2" width="13.28515625" style="11" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" style="11" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" style="11" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" style="11" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" style="11" customWidth="1"/>
+    <col min="12" max="12" width="14.7109375" style="11" customWidth="1"/>
+    <col min="13" max="13" width="9.140625" style="11"/>
+    <col min="14" max="14" width="11.7109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.85546875" style="11" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" style="11"/>
+    <col min="17" max="17" width="11.7109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.85546875" style="11" customWidth="1"/>
+    <col min="19" max="21" width="9.140625" style="11"/>
+    <col min="22" max="22" width="12.140625" style="11" customWidth="1"/>
+    <col min="23" max="23" width="14.140625" style="11" customWidth="1"/>
+    <col min="24" max="16384" width="9.140625" style="11"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="28" t="s">
         <v>41</v>
       </c>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="W2" s="27"/>
     </row>
-    <row r="3" spans="2:23" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:23" ht="45" x14ac:dyDescent="0.25">
       <c r="B3" s="6" t="s">
         <v>42</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:23" ht="15" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
         <v>75</v>
       </c>
@@ -1713,7 +1713,7 @@
         <v>98.018918918918899</v>
       </c>
     </row>
-    <row r="5" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:23" ht="15" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
         <v>150</v>
       </c>
@@ -1752,8 +1752,8 @@
         <v>46</v>
       </c>
       <c r="R5" s="8">
-        <f>AVERAGE(H81:H114)</f>
-        <v>106.59</v>
+        <f>AVERAGE(G81:G114)</f>
+        <v>161.5</v>
       </c>
       <c r="V5" s="6" t="s">
         <v>34</v>
@@ -1763,7 +1763,7 @@
         <v>52.299254158004175</v>
       </c>
     </row>
-    <row r="6" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:23" ht="15" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
         <v>225</v>
       </c>
@@ -1803,17 +1803,17 @@
       </c>
       <c r="R6" s="8">
         <f>ABS(R4-R5)</f>
-        <v>51.552857142857135</v>
+        <v>3.3571428571428612</v>
       </c>
       <c r="V6" s="6" t="s">
         <v>54</v>
       </c>
       <c r="W6" s="8">
         <f>AVERAGE(R4:R5)-W4</f>
-        <v>34.347509652509672</v>
-      </c>
-    </row>
-    <row r="7" spans="2:23" x14ac:dyDescent="0.3">
+        <v>61.802509652509656</v>
+      </c>
+    </row>
+    <row r="7" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
         <v>300</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>145.86000000000001</v>
       </c>
     </row>
-    <row r="8" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
         <v>375</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>146.52000000000001</v>
       </c>
     </row>
-    <row r="9" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
         <v>450</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>525</v>
       </c>
@@ -1904,7 +1904,7 @@
         <v>148.5</v>
       </c>
     </row>
-    <row r="11" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <v>600</v>
       </c>
@@ -1926,7 +1926,7 @@
         <v>147.18</v>
       </c>
     </row>
-    <row r="12" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <v>675</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>143.88</v>
       </c>
     </row>
-    <row r="13" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <v>750</v>
       </c>
@@ -1970,7 +1970,7 @@
         <v>144.54000000000002</v>
       </c>
     </row>
-    <row r="14" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <v>825</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>143.88</v>
       </c>
     </row>
-    <row r="15" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <v>900</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>143.88</v>
       </c>
     </row>
-    <row r="16" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <v>975</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>144.54000000000002</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <v>1050</v>
       </c>
@@ -2058,7 +2058,7 @@
         <v>144.54000000000002</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <v>1125</v>
       </c>
@@ -2080,7 +2080,7 @@
         <v>143.88</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <v>1200</v>
       </c>
@@ -2102,7 +2102,7 @@
         <v>147.84</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <v>1275</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>147.18</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <v>1350</v>
       </c>
@@ -2146,7 +2146,7 @@
         <v>144.54000000000002</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <v>1425</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>145.20000000000002</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <v>1500</v>
       </c>
@@ -2190,7 +2190,7 @@
         <v>143.88</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <v>1575</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>143.88</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <v>1650</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>143.88</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <v>1725</v>
       </c>
@@ -2256,7 +2256,7 @@
         <v>143.88</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" s="3">
         <v>1800</v>
       </c>
@@ -2278,7 +2278,7 @@
         <v>171.6</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" s="3">
         <v>1875</v>
       </c>
@@ -2300,7 +2300,7 @@
         <v>172.26000000000002</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" s="3">
         <v>1950</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>170.94</v>
       </c>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" s="3">
         <v>2025</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>146.52000000000001</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" s="3">
         <v>2100</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>162.36000000000001</v>
       </c>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" s="3">
         <v>2175</v>
       </c>
@@ -2388,7 +2388,7 @@
         <v>150.48000000000002</v>
       </c>
     </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B33" s="3">
         <v>2250</v>
       </c>
@@ -2410,7 +2410,7 @@
         <v>144.54000000000002</v>
       </c>
     </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B34" s="3">
         <v>2325</v>
       </c>
@@ -2432,7 +2432,7 @@
         <v>167.64000000000001</v>
       </c>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="3">
         <v>2400</v>
       </c>
@@ -2454,7 +2454,7 @@
         <v>148.5</v>
       </c>
     </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B36" s="3">
         <v>2475</v>
       </c>
@@ -2476,7 +2476,7 @@
         <v>145.86000000000001</v>
       </c>
     </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="3">
         <v>2550</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>159.72</v>
       </c>
     </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="3">
         <v>2625</v>
       </c>
@@ -2520,7 +2520,7 @@
         <v>170.94</v>
       </c>
     </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B39" s="3">
         <v>2700</v>
       </c>
@@ -2542,7 +2542,7 @@
         <v>146.52000000000001</v>
       </c>
     </row>
-    <row r="40" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B40" s="3">
         <v>2775</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>170.94</v>
       </c>
     </row>
-    <row r="41" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B41" s="3">
         <v>2850</v>
       </c>
@@ -2586,7 +2586,7 @@
         <v>170.28</v>
       </c>
     </row>
-    <row r="42" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B42" s="3">
         <v>2925</v>
       </c>
@@ -2608,7 +2608,7 @@
         <v>144.54000000000002</v>
       </c>
     </row>
-    <row r="43" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B43" s="3">
         <v>3000</v>
       </c>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="J43" s="12"/>
     </row>
-    <row r="44" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B44" s="3">
         <v>3075</v>
       </c>
@@ -2659,7 +2659,7 @@
         <v>97.02000000000001</v>
       </c>
     </row>
-    <row r="45" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B45" s="3">
         <v>3150</v>
       </c>
@@ -2681,7 +2681,7 @@
         <v>98.34</v>
       </c>
     </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" s="3">
         <v>3225</v>
       </c>
@@ -2703,7 +2703,7 @@
         <v>96.36</v>
       </c>
     </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B47" s="3">
         <v>3300</v>
       </c>
@@ -2725,7 +2725,7 @@
         <v>97.02000000000001</v>
       </c>
     </row>
-    <row r="48" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B48" s="3">
         <v>3375</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>96.36</v>
       </c>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B49" s="3">
         <v>3450</v>
       </c>
@@ -2769,7 +2769,7 @@
         <v>98.34</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="3">
         <v>3525</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="3">
         <v>3600</v>
       </c>
@@ -2813,7 +2813,7 @@
         <v>97.68</v>
       </c>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B52" s="3">
         <v>3675</v>
       </c>
@@ -2835,7 +2835,7 @@
         <v>97.02000000000001</v>
       </c>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B53" s="3">
         <v>3750</v>
       </c>
@@ -2857,7 +2857,7 @@
         <v>97.68</v>
       </c>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B54" s="3">
         <v>3825</v>
       </c>
@@ -2879,7 +2879,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B55" s="3">
         <v>3900</v>
       </c>
@@ -2901,7 +2901,7 @@
         <v>98.34</v>
       </c>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B56" s="3">
         <v>3975</v>
       </c>
@@ -2923,7 +2923,7 @@
         <v>98.34</v>
       </c>
     </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B57" s="3">
         <v>4050</v>
       </c>
@@ -2945,7 +2945,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B58" s="3">
         <v>4125</v>
       </c>
@@ -2967,7 +2967,7 @@
         <v>95.04</v>
       </c>
     </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B59" s="3">
         <v>4200</v>
       </c>
@@ -2989,7 +2989,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B60" s="3">
         <v>4275</v>
       </c>
@@ -3011,7 +3011,7 @@
         <v>96.36</v>
       </c>
     </row>
-    <row r="61" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B61" s="3">
         <v>4350</v>
       </c>
@@ -3033,7 +3033,7 @@
         <v>97.02000000000001</v>
       </c>
     </row>
-    <row r="62" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B62" s="3">
         <v>4425</v>
       </c>
@@ -3055,7 +3055,7 @@
         <v>97.02000000000001</v>
       </c>
     </row>
-    <row r="63" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B63" s="3">
         <v>4500</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>97.68</v>
       </c>
     </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B64" s="3">
         <v>4575</v>
       </c>
@@ -3099,7 +3099,7 @@
         <v>96.36</v>
       </c>
     </row>
-    <row r="65" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B65" s="3">
         <v>4650</v>
       </c>
@@ -3121,7 +3121,7 @@
         <v>97.68</v>
       </c>
     </row>
-    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B66" s="3">
         <v>4725</v>
       </c>
@@ -3143,7 +3143,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="67" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B67" s="3">
         <v>4800</v>
       </c>
@@ -3165,7 +3165,7 @@
         <v>97.68</v>
       </c>
     </row>
-    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B68" s="3">
         <v>4875</v>
       </c>
@@ -3187,7 +3187,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="69" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B69" s="3">
         <v>4950</v>
       </c>
@@ -3209,7 +3209,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="70" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B70" s="3">
         <v>5025</v>
       </c>
@@ -3231,7 +3231,7 @@
         <v>95.04</v>
       </c>
     </row>
-    <row r="71" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B71" s="3">
         <v>5100</v>
       </c>
@@ -3253,7 +3253,7 @@
         <v>97.68</v>
       </c>
     </row>
-    <row r="72" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B72" s="3">
         <v>5175</v>
       </c>
@@ -3275,7 +3275,7 @@
         <v>97.68</v>
       </c>
     </row>
-    <row r="73" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B73" s="3">
         <v>5250</v>
       </c>
@@ -3297,7 +3297,7 @@
         <v>96.36</v>
       </c>
     </row>
-    <row r="74" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B74" s="3">
         <v>5325</v>
       </c>
@@ -3319,7 +3319,7 @@
         <v>97.68</v>
       </c>
     </row>
-    <row r="75" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B75" s="3">
         <v>5400</v>
       </c>
@@ -3341,7 +3341,7 @@
         <v>97.68</v>
       </c>
     </row>
-    <row r="76" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B76" s="3">
         <v>5475</v>
       </c>
@@ -3363,7 +3363,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="77" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B77" s="3">
         <v>5550</v>
       </c>
@@ -3385,7 +3385,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="78" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B78" s="3">
         <v>5625</v>
       </c>
@@ -3407,7 +3407,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="79" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B79" s="3">
         <v>5700</v>
       </c>
@@ -3429,7 +3429,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="80" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B80" s="3">
         <v>5775</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>98.34</v>
       </c>
     </row>
-    <row r="81" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B81" s="3">
         <v>5850</v>
       </c>
@@ -3479,7 +3479,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="82" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B82" s="3">
         <v>5925</v>
       </c>
@@ -3501,7 +3501,7 @@
         <v>103.62</v>
       </c>
     </row>
-    <row r="83" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B83" s="3">
         <v>6000</v>
       </c>
@@ -3523,7 +3523,7 @@
         <v>102.96000000000001</v>
       </c>
     </row>
-    <row r="84" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B84" s="3">
         <v>6075</v>
       </c>
@@ -3545,7 +3545,7 @@
         <v>100.98</v>
       </c>
     </row>
-    <row r="85" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B85" s="3">
         <v>6150</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>102.30000000000001</v>
       </c>
     </row>
-    <row r="86" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B86" s="3">
         <v>6225</v>
       </c>
@@ -3589,7 +3589,7 @@
         <v>102.96000000000001</v>
       </c>
     </row>
-    <row r="87" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B87" s="3">
         <v>6300</v>
       </c>
@@ -3611,7 +3611,7 @@
         <v>101.64</v>
       </c>
     </row>
-    <row r="88" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B88" s="3">
         <v>6375</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>102.96000000000001</v>
       </c>
     </row>
-    <row r="89" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D89" s="19">
         <f>C89*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3649,7 +3649,7 @@
         <v>102.30000000000001</v>
       </c>
     </row>
-    <row r="90" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D90" s="19">
         <f>C90*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3665,7 +3665,7 @@
         <v>99.660000000000011</v>
       </c>
     </row>
-    <row r="91" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D91" s="19">
         <f>C91*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3681,7 +3681,7 @@
         <v>99.660000000000011</v>
       </c>
     </row>
-    <row r="92" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D92" s="19">
         <f>C92*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3697,7 +3697,7 @@
         <v>105.60000000000001</v>
       </c>
     </row>
-    <row r="93" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D93" s="19">
         <f>C93*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3713,7 +3713,7 @@
         <v>100.98</v>
       </c>
     </row>
-    <row r="94" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D94" s="19">
         <f>C94*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3729,7 +3729,7 @@
         <v>99.660000000000011</v>
       </c>
     </row>
-    <row r="95" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D95" s="19">
         <f>C95*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3745,7 +3745,7 @@
         <v>106.26</v>
       </c>
     </row>
-    <row r="96" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D96" s="19">
         <f>C96*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3761,7 +3761,7 @@
         <v>101.64</v>
       </c>
     </row>
-    <row r="97" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D97" s="19">
         <f>C97*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3777,7 +3777,7 @@
         <v>101.64</v>
       </c>
     </row>
-    <row r="98" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D98" s="19">
         <f>C98*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3793,7 +3793,7 @@
         <v>129.36000000000001</v>
       </c>
     </row>
-    <row r="99" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D99" s="19">
         <f>C99*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3809,7 +3809,7 @@
         <v>126.72</v>
       </c>
     </row>
-    <row r="100" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D100" s="19">
         <f>C100*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3825,7 +3825,7 @@
         <v>127.38000000000001</v>
       </c>
     </row>
-    <row r="101" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D101" s="19">
         <f>C101*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3841,7 +3841,7 @@
         <v>128.04</v>
       </c>
     </row>
-    <row r="102" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D102" s="19">
         <f>C102*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3857,7 +3857,7 @@
         <v>125.4</v>
       </c>
     </row>
-    <row r="103" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D103" s="19">
         <f>C103*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3873,7 +3873,7 @@
         <v>126.06</v>
       </c>
     </row>
-    <row r="104" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D104" s="19">
         <f>C104*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3889,7 +3889,7 @@
         <v>112.86</v>
       </c>
     </row>
-    <row r="105" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D105" s="19">
         <f>C105*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3905,7 +3905,7 @@
         <v>101.64</v>
       </c>
     </row>
-    <row r="106" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D106" s="19">
         <f>C106*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3921,7 +3921,7 @@
         <v>100.32000000000001</v>
       </c>
     </row>
-    <row r="107" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D107" s="19">
         <f>C107*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3937,7 +3937,7 @@
         <v>101.64</v>
       </c>
     </row>
-    <row r="108" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D108" s="19">
         <f>C108*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3953,7 +3953,7 @@
         <v>101.64</v>
       </c>
     </row>
-    <row r="109" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D109" s="19">
         <f>C109*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3969,7 +3969,7 @@
         <v>101.64</v>
       </c>
     </row>
-    <row r="110" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D110" s="19">
         <f>C110*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -3985,7 +3985,7 @@
         <v>104.28</v>
       </c>
     </row>
-    <row r="111" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D111" s="19">
         <f>C111*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -4001,7 +4001,7 @@
         <v>99.660000000000011</v>
       </c>
     </row>
-    <row r="112" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D112" s="19">
         <f>C112*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -4017,7 +4017,7 @@
         <v>99.660000000000011</v>
       </c>
     </row>
-    <row r="113" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D113" s="19">
         <f>C113*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -4033,7 +4033,7 @@
         <v>102.30000000000001</v>
       </c>
     </row>
-    <row r="114" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D114" s="19">
         <f>C114*'SYS INFO'!$C$9</f>
         <v>0</v>
@@ -4066,23 +4066,23 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5797DBD1-C226-49A6-AAF8-43F72E436050}">
   <dimension ref="B2:L24"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="2"/>
-    <col min="2" max="2" width="6.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.21875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" style="2" customWidth="1"/>
-    <col min="5" max="6" width="8.88671875" style="2"/>
-    <col min="7" max="7" width="20.5546875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="21.5546875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="2"/>
-    <col min="10" max="10" width="15.33203125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="8.88671875" style="2"/>
-    <col min="12" max="12" width="14.109375" style="2" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="8.85546875" style="2"/>
+    <col min="2" max="2" width="6.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" style="2" customWidth="1"/>
+    <col min="5" max="6" width="8.85546875" style="2"/>
+    <col min="7" max="7" width="20.5703125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" style="2"/>
+    <col min="10" max="10" width="15.28515625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" style="2"/>
+    <col min="12" max="12" width="14.140625" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="29" t="s">
         <v>69</v>
       </c>
@@ -4101,7 +4101,7 @@
       <c r="K2" s="30"/>
       <c r="L2" s="30"/>
     </row>
-    <row r="3" spans="2:12" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" ht="30" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
         <v>0</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" ht="15" x14ac:dyDescent="0.2">
       <c r="B4" s="3">
         <v>1</v>
       </c>
@@ -4161,7 +4161,7 @@
         <v>64.267500000000013</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" ht="15" x14ac:dyDescent="0.2">
       <c r="B5" s="3">
         <v>2</v>
       </c>
@@ -4194,7 +4194,7 @@
         <v>78.719144361702121</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" ht="15" x14ac:dyDescent="0.2">
       <c r="B6" s="3">
         <v>3</v>
       </c>
@@ -4227,7 +4227,7 @@
         <v>14.451644361702108</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B7" s="3">
         <v>4</v>
       </c>
@@ -4249,7 +4249,7 @@
         <v>59.711730638297865</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B8" s="3">
         <v>5</v>
       </c>
@@ -4271,7 +4271,7 @@
         <v>60.082980638297862</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" ht="15" x14ac:dyDescent="0.2">
       <c r="C10" s="6" t="s">
         <v>12</v>
       </c>
@@ -4287,19 +4287,19 @@
         <v>60.004605638297868</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.2">
       <c r="G12" s="18" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="2:12" ht="22.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" ht="22.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F14" s="29" t="s">
         <v>88</v>
       </c>
       <c r="G14" s="29"/>
       <c r="H14" s="29"/>
     </row>
-    <row r="15" spans="2:12" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" ht="30" x14ac:dyDescent="0.2">
       <c r="F15" s="4" t="s">
         <v>0</v>
       </c>
@@ -4310,7 +4310,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.2">
       <c r="F16" s="3">
         <v>1</v>
       </c>
@@ -4322,7 +4322,7 @@
         <v>18.337980638297871</v>
       </c>
     </row>
-    <row r="17" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="6:8" x14ac:dyDescent="0.2">
       <c r="F17" s="3">
         <v>2</v>
       </c>
@@ -4334,7 +4334,7 @@
         <v>18.358605638297867</v>
       </c>
     </row>
-    <row r="18" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="6:8" x14ac:dyDescent="0.2">
       <c r="F18" s="3">
         <v>3</v>
       </c>
@@ -4346,7 +4346,7 @@
         <v>18.317355638297869</v>
       </c>
     </row>
-    <row r="19" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="6:8" x14ac:dyDescent="0.2">
       <c r="F19" s="3">
         <v>4</v>
       </c>
@@ -4358,7 +4358,7 @@
         <v>18.255480638297872</v>
       </c>
     </row>
-    <row r="20" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="6:8" x14ac:dyDescent="0.2">
       <c r="F20" s="3">
         <v>5</v>
       </c>
@@ -4370,7 +4370,7 @@
         <v>18.193605638297871</v>
       </c>
     </row>
-    <row r="22" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="6:8" ht="15" x14ac:dyDescent="0.2">
       <c r="G22" s="6" t="s">
         <v>12</v>
       </c>
@@ -4379,7 +4379,7 @@
         <v>18.292605638297868</v>
       </c>
     </row>
-    <row r="24" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="6:8" x14ac:dyDescent="0.2">
       <c r="G24" s="18" t="s">
         <v>75</v>
       </c>
@@ -4398,16 +4398,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECF03045-3C2D-471C-842A-3F9D869D102D}">
   <dimension ref="B2:F20"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="11"/>
-    <col min="2" max="4" width="16.109375" style="11" customWidth="1"/>
-    <col min="5" max="5" width="39.88671875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="23.21875" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="11"/>
+    <col min="1" max="1" width="9.140625" style="11"/>
+    <col min="2" max="4" width="16.140625" style="11" customWidth="1"/>
+    <col min="5" max="5" width="39.85546875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="11"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="14" t="s">
         <v>2</v>
       </c>
@@ -4421,7 +4421,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>35</v>
       </c>
@@ -4436,7 +4436,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>36</v>
       </c>
@@ -4449,7 +4449,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>37</v>
       </c>
@@ -4464,7 +4464,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>38</v>
       </c>
@@ -4480,7 +4480,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>71</v>
       </c>
@@ -4498,7 +4498,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>82</v>
       </c>
@@ -4516,7 +4516,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>85</v>
       </c>
@@ -4535,7 +4535,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>33</v>
       </c>
@@ -4550,7 +4550,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>34</v>
       </c>
@@ -4563,33 +4563,33 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>57</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="7">
         <f>'Camera Test'!W6</f>
-        <v>34.347509652509672</v>
+        <v>61.802509652509656</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>63</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="7">
         <f>SUM(D3:D12)*('SYS INFO'!$C$8)</f>
-        <v>137.12315634081278</v>
+        <v>151.26664118929762</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
         <v>65</v>
       </c>
@@ -4602,7 +4602,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>68</v>
       </c>
@@ -4615,7 +4615,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
         <v>87</v>
       </c>
@@ -4628,16 +4628,16 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:5" ht="15" x14ac:dyDescent="0.25">
       <c r="C17" s="21" t="s">
         <v>64</v>
       </c>
       <c r="D17" s="22">
         <f>SUM(D3:D13)-D8-D9</f>
-        <v>371.70590100239048</v>
-      </c>
-    </row>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.3">
+        <v>413.30438585087524</v>
+      </c>
+    </row>
+    <row r="18" spans="3:5" ht="15" x14ac:dyDescent="0.25">
       <c r="C18" s="14" t="s">
         <v>66</v>
       </c>
@@ -4646,7 +4646,7 @@
         <v>149.14542553191492</v>
       </c>
     </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:5" ht="15" x14ac:dyDescent="0.25">
       <c r="C19" s="14" t="s">
         <v>84</v>
       </c>
@@ -4658,7 +4658,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="3:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="C20" s="14" t="s">
         <v>86</v>
       </c>

</xml_diff>